<commit_message>
feat: add guided spreadsheet template
</commit_message>
<xml_diff>
--- a/docs/sample-upload-template.xlsx
+++ b/docs/sample-upload-template.xlsx
@@ -3,8 +3,12 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="sample" sheetId="1" r:id="rId1"/>
+    <sheet name="데이터" sheetId="1" r:id="rId1"/>
+    <sheet name="사용법" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'데이터'!A1:E4</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -398,6 +402,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E4"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -407,7 +418,7 @@
         <v>이름</v>
       </c>
       <c r="C1" t="str">
-        <v>값</v>
+        <v>대표값</v>
       </c>
       <c r="D1" t="str">
         <v>분류</v>
@@ -418,58 +429,169 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>세종특별자치시 도움6로 11</v>
+        <v>서울 서초구 반포대로 58</v>
       </c>
       <c r="B2" t="str">
-        <v>정부세종청사</v>
+        <v>예시복지관</v>
       </c>
       <c r="C2">
-        <v>100</v>
+        <v>48</v>
       </c>
       <c r="D2" t="str">
-        <v>행정</v>
+        <v>복지</v>
       </c>
       <c r="E2" t="str">
-        <v>중앙행정기관</v>
+        <v>담당부서, 비고</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>서울특별시 중구 세종대로 110</v>
+        <v>부산 해운대구 센텀로 10</v>
       </c>
       <c r="B3" t="str">
-        <v>서울시청</v>
+        <v>예시청년센터</v>
       </c>
       <c r="C3">
-        <v>80</v>
+        <v>36</v>
       </c>
       <c r="D3" t="str">
-        <v>지자체</v>
+        <v>청년</v>
       </c>
       <c r="E3" t="str">
-        <v>광역자치단체</v>
+        <v>운영 중</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>대전광역시 서구 청사로 189</v>
+        <v>대전 유성구 대학로 99</v>
       </c>
       <c r="B4" t="str">
-        <v>정부대전청사</v>
+        <v>예시상담소</v>
       </c>
       <c r="C4">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="D4" t="str">
-        <v>행정</v>
+        <v>점검</v>
       </c>
       <c r="E4" t="str">
-        <v>행정기관 집적지</v>
+        <v>점검 예정</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E4"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B13"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="68.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>GonpunClaw PolicyMap 템플릿 사용법</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>핵심 원칙</v>
+      </c>
+      <c r="B3" t="str">
+        <v>한 행은 지도에 표시될 위치 1개입니다.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>시트</v>
+      </c>
+      <c r="B4" t="str">
+        <v>첫 번째 시트만 읽습니다. 데이터 시트 이름은 바꾸지 않는 편이 좋습니다.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>A열 주소</v>
+      </c>
+      <c r="B5" t="str">
+        <v>필수입니다. 도로명주소처럼 가능한 정확하게 입력하세요.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>B열 이름</v>
+      </c>
+      <c r="B6" t="str">
+        <v>지도와 표에 표시할 위치 이름입니다.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>C열 대표값</v>
+      </c>
+      <c r="B7" t="str">
+        <v>위치 1개에 붙일 숫자 1개입니다. 필터와 표에 사용됩니다.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>D열 분류</v>
+      </c>
+      <c r="B8" t="str">
+        <v>복지, 청년, 점검처럼 묶어 볼 기준입니다.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>E열 이후</v>
+      </c>
+      <c r="B9" t="str">
+        <v>E열 이후는 공개 지도 팝업에 추가 정보로 표시됩니다.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>주의</v>
+      </c>
+      <c r="B10" t="str">
+        <v>개인정보나 민감정보가 들어 있는 열은 업로드 전에 제거하세요.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>예시</v>
+      </c>
+      <c r="B12" t="str">
+        <v>서울 서초구 반포대로 58 / 예시복지관 / 48 / 복지 / 담당부서, 비고</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>결과</v>
+      </c>
+      <c r="B13" t="str">
+        <v>위 예시 행은 지도에서 예시복지관 위치 1개로 표시됩니다.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>